<commit_message>
Non-subsantial but important robustness additions
Added individual synthetic DIDs for each country. Created the citation mamager for the finalization of the manuscript before editage.
</commit_message>
<xml_diff>
--- a/Statistical_documentation_in_R/Present_ value_simulations/betas_saturated_model.xlsx
+++ b/Statistical_documentation_in_R/Present_ value_simulations/betas_saturated_model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stoycho.rusinov\Documents\GitHub\Estimating_price_elasticity\Statistical_documentation_in_R\Present_ value_simulations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FABE23-7DA7-41C4-B4D4-8FF86C6B3D4E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6732507-91A3-460E-AF35-80E756CC6532}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10380" xr2:uid="{199D723B-9A26-436A-828C-653175FE4DF6}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10380" activeTab="2" xr2:uid="{199D723B-9A26-436A-828C-653175FE4DF6}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="41">
   <si>
     <t>Country</t>
   </si>
@@ -142,13 +142,16 @@
     <t>Term</t>
   </si>
   <si>
-    <t xml:space="preserve">Controls </t>
-  </si>
-  <si>
     <t xml:space="preserve">Term </t>
   </si>
   <si>
     <t xml:space="preserve">Constant </t>
+  </si>
+  <si>
+    <t>Control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">term </t>
   </si>
 </sst>
 </file>
@@ -172,18 +175,12 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -224,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -232,15 +229,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,7 +574,7 @@
       </c>
       <c r="C2">
         <f>VLOOKUP(A2,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.52253281187205503</v>
+        <v>-0.503790953780059</v>
       </c>
       <c r="D2">
         <f>VLOOKUP(A2,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -602,7 +591,7 @@
       </c>
       <c r="C3">
         <f>VLOOKUP(A3,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.58881474953060198</v>
+        <v>-0.57561060819490195</v>
       </c>
       <c r="D3">
         <f>VLOOKUP(A3,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -619,7 +608,7 @@
       </c>
       <c r="C4">
         <f>VLOOKUP(A4,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.7500224026120099</v>
+        <v>-1.78417059468777</v>
       </c>
       <c r="D4">
         <f>VLOOKUP(A4,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -636,7 +625,7 @@
       </c>
       <c r="C5">
         <f>VLOOKUP(A5,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.5039661484504001</v>
+        <v>-1.5329456248967499</v>
       </c>
       <c r="D5">
         <f>VLOOKUP(A5,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -653,7 +642,7 @@
       </c>
       <c r="C6">
         <f>VLOOKUP(A6,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.91761150119939405</v>
+        <v>-0.94501847818830298</v>
       </c>
       <c r="D6">
         <f>VLOOKUP(A6,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -670,7 +659,7 @@
       </c>
       <c r="C7">
         <f>VLOOKUP(A7,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.0850792485018901</v>
+        <v>-1.07565711034427</v>
       </c>
       <c r="D7">
         <f>VLOOKUP(A7,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -687,7 +676,7 @@
       </c>
       <c r="C8">
         <f>VLOOKUP(A8,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.0320420194351301</v>
+        <v>-1.0301060798322601</v>
       </c>
       <c r="D8">
         <f>VLOOKUP(A8,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -704,7 +693,7 @@
       </c>
       <c r="C9">
         <f>VLOOKUP(A9,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.42585548921212</v>
+        <v>-1.4075162526001099</v>
       </c>
       <c r="D9">
         <f>VLOOKUP(A9,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -721,7 +710,7 @@
       </c>
       <c r="C10">
         <f>VLOOKUP(A10,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.7120798527741501</v>
+        <v>-1.6216422891201301</v>
       </c>
       <c r="D10">
         <f>VLOOKUP(A10,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -738,7 +727,7 @@
       </c>
       <c r="C11">
         <f>VLOOKUP(A11,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.56116384477579395</v>
+        <v>-0.53652430994564804</v>
       </c>
       <c r="D11">
         <f>VLOOKUP(A11,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -755,7 +744,7 @@
       </c>
       <c r="C12">
         <f>VLOOKUP(A12,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.60269935069783398</v>
+        <v>-0.58277125268367203</v>
       </c>
       <c r="D12">
         <f>VLOOKUP(A12,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -772,7 +761,7 @@
       </c>
       <c r="C13">
         <f>VLOOKUP(A13,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.74723026677037296</v>
+        <v>-0.71947138260508403</v>
       </c>
       <c r="D13">
         <f>VLOOKUP(A13,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -789,7 +778,7 @@
       </c>
       <c r="C14">
         <f>VLOOKUP(A14,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.00784479539697</v>
+        <v>-1.02268425869302</v>
       </c>
       <c r="D14">
         <f>VLOOKUP(A14,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -806,7 +795,7 @@
       </c>
       <c r="C15">
         <f>VLOOKUP(A15,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.84259563933272497</v>
+        <v>-0.81079323871487197</v>
       </c>
       <c r="D15">
         <f>VLOOKUP(A15,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -823,7 +812,7 @@
       </c>
       <c r="C16">
         <f>VLOOKUP(A16,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.3877153397395701</v>
+        <v>-1.3904913497439999</v>
       </c>
       <c r="D16">
         <f>VLOOKUP(A16,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -840,7 +829,7 @@
       </c>
       <c r="C17">
         <f>VLOOKUP(A17,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-2.1334699586950201</v>
+        <v>-2.1660399744893502</v>
       </c>
       <c r="D17">
         <f>VLOOKUP(A17,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -857,7 +846,7 @@
       </c>
       <c r="C18">
         <f>VLOOKUP(A18,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.58971650808602505</v>
+        <v>-0.57603562801806196</v>
       </c>
       <c r="D18">
         <f>VLOOKUP(A18,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -874,7 +863,7 @@
       </c>
       <c r="C19">
         <f>VLOOKUP(A19,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.517079079002839</v>
+        <v>-0.52892439215107301</v>
       </c>
       <c r="D19">
         <f>VLOOKUP(A19,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -891,7 +880,7 @@
       </c>
       <c r="C20">
         <f>VLOOKUP(A20,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.53118369958342704</v>
+        <v>-0.52702850261561396</v>
       </c>
       <c r="D20">
         <f>VLOOKUP(A20,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -908,7 +897,7 @@
       </c>
       <c r="C21">
         <f>VLOOKUP(A21,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.5092784317056001</v>
+        <v>-1.52760392501248</v>
       </c>
       <c r="D21">
         <f>VLOOKUP(A21,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -925,7 +914,7 @@
       </c>
       <c r="C22">
         <f>VLOOKUP(A22,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.90214523845726202</v>
+        <v>-0.83612033855998502</v>
       </c>
       <c r="D22">
         <f>VLOOKUP(A22,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -942,7 +931,7 @@
       </c>
       <c r="C23">
         <f>VLOOKUP(A23,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.5947580894711899</v>
+        <v>-1.6001173391912</v>
       </c>
       <c r="D23">
         <f>VLOOKUP(A23,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -959,7 +948,7 @@
       </c>
       <c r="C24">
         <f>VLOOKUP(A24,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.40384996280401</v>
+        <v>-1.39755782045907</v>
       </c>
       <c r="D24">
         <f>VLOOKUP(A24,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -976,7 +965,7 @@
       </c>
       <c r="C25">
         <f>VLOOKUP(A25,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-1.2207771640338001</v>
+        <v>-1.1788745227473101</v>
       </c>
       <c r="D25">
         <f>VLOOKUP(A25,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -993,7 +982,7 @@
       </c>
       <c r="C26">
         <f>VLOOKUP(A26,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.50905610951238001</v>
+        <v>-0.47498173216436002</v>
       </c>
       <c r="D26">
         <f>VLOOKUP(A26,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -1010,7 +999,7 @@
       </c>
       <c r="C27">
         <f>VLOOKUP(A27,TWFE_CONTROLS!$A$1:$B$30,2,FALSE)</f>
-        <v>-0.978668873912933</v>
+        <v>-0.92763206000377596</v>
       </c>
       <c r="D27">
         <f>VLOOKUP(A27,Pooled!$A$1:$B$28,2,FALSE)</f>
@@ -1028,14 +1017,14 @@
   <dimension ref="A1:G27"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.44140625" customWidth="1"/>
+    <col min="1" max="1" width="12.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -1055,600 +1044,600 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3">
         <v>-0.54852831529282597</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>5.3467133275019299E-2</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>-10.259279395445899</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>2.8904300786899701E-6</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <v>-0.66948531725433502</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="3">
         <v>-0.42758320022959301</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>-0.60265118871781398</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>6.6890441900966699E-2</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>-9.0096150517170202</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>8.4637891956509398E-6</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>-0.75397382443596195</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>-0.45134043989794398</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>-1.88714028053297</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>0.13227254971833599</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>-14.2671040060893</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>1.7416340389940201E-7</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>-2.1863675197690302</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>-1.5879249281951999</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>-1.65473875502575</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>0.109941116750136</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>-15.0511905589939</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>1.09520756228172E-7</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>-1.90344878321724</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="3">
         <v>-1.4060406137325401</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>-0.90215690028786599</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>6.8075532379029996E-2</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>-13.252380293024499</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>3.2915851283455998E-7</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>-1.0561603969195299</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>-0.748165290554482</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>-1.1371955365404101</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>5.6221398163693502E-2</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>-20.2272002677431</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>8.2183524438405404E-9</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <v>-1.2643831185480801</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="3">
         <v>-1.01001984143102</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>-1.0464974377475</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>0.110553592437794</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>-9.4660278161968296</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>5.6389900372636702E-6</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <v>-1.2965929822028699</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="3">
         <v>-0.79641378019041498</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>-1.4474385643897401</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>0.11899090479088401</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>-12.1643289491969</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>6.8569548568021996E-7</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>-1.71662063541942</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <v>-1.17826838025835</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="3">
         <v>-1.75634080420609</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>0.20804537696209499</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>-8.4421330255045</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>1.4366154137722E-5</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>-2.2269780873370899</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>-1.2857154079733799</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="3">
         <v>-0.59709956840556899</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>6.2239968720100403E-2</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>-9.5936023769541698</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>5.0485996253519998E-6</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>-0.73790210290721903</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <v>-0.45630892080219698</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="3">
         <v>-0.68149440447415999</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>7.2888343121077004E-2</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>-9.3499223434293093</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>6.2428939193372297E-6</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>-0.84638523539913701</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>-0.51661546044746198</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="3">
         <v>-0.86574363247956398</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>7.8845788640573095E-2</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>-10.9802893833089</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>1.63446404840163E-6</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>-1.0441111414584501</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="3">
         <v>-0.68738801039895803</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="3">
         <v>-1.1144617208190799</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>7.7838449110645705E-2</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>-14.317701303170001</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <v>1.6890823877634501E-7</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="3">
         <v>-1.2905504694649701</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="3">
         <v>-0.93838485907147196</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="3">
         <v>-0.92503071686511495</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>0.11325856897063399</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="3">
         <v>-8.1674761452628104</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>1.8751006902026799E-5</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="3">
         <v>-1.1812453433594501</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <v>-0.66882797726906096</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="3">
         <v>-1.51151031782695</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <v>0.128184277456144</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>-11.791744598265799</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <v>8.9369534154202703E-7</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="3">
         <v>-1.80148924268162</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="3">
         <v>-1.2215432798705601</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="3">
         <v>-2.1731071022163002</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>0.28010211549720998</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>-7.7582885863176996</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <v>2.8259097861567101E-5</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="3">
         <v>-2.8067480525523898</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="3">
         <v>-1.5394780387785001</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="3">
         <v>-0.492889178451345</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="3">
         <v>4.7435761946085203E-2</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>-10.3907917081779</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <v>2.5983892145060802E-6</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="3">
         <v>-0.60020227055961095</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="3">
         <v>-0.38558797324135702</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="3">
         <v>-0.36167297288073402</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="3">
         <v>4.5339212630366402E-2</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>-7.9771768265696501</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <v>2.2645699902786299E-5</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="3">
         <v>-0.46424334093728697</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="3">
         <v>-0.25911449172245898</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="3">
         <v>-0.534966490387353</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="3">
         <v>2.42064072544547E-2</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>-22.100447547334401</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <v>3.7567958910538196E-9</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="3">
         <v>-0.58973113139276601</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="3">
         <v>-0.48021373628021602</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="3">
         <v>-1.66827531130462</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="3">
         <v>0.15070707857215501</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <v>-11.0696940751528</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <v>1.5263966707082899E-6</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="3">
         <v>-2.0092043520301601</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="3">
         <v>-1.3273581574773801</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="3">
         <v>-0.93916309417618304</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="3">
         <v>0.35342907395453099</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="3">
         <v>-2.6573055439863098</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="3">
         <v>2.6161065918485701E-2</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="3">
         <v>-1.7386811488127001</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="3">
         <v>-0.139656926437944</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="3">
         <v>-1.7114266042599799</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="3">
         <v>0.13749724235369701</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <v>-12.447031797966099</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="3">
         <v>5.6352972987097596E-7</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="3">
         <v>-2.0224729193645401</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="3">
         <v>-1.4003921760536999</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="3">
         <v>-1.51631980729154</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="3">
         <v>0.120029805159765</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="3">
         <v>-12.6329102069472</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <v>4.9640047382324196E-7</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="3">
         <v>-1.78785203423211</v>
       </c>
-      <c r="G24" s="4">
+      <c r="G24" s="3">
         <v>-1.24479946724924</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="3">
         <v>-1.2795484913805499</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <v>0.122303206789315</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <v>-10.462149508752599</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="3">
         <v>2.4536643556643401E-6</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="3">
         <v>-1.55622351010134</v>
       </c>
-      <c r="G25" s="4">
+      <c r="G25" s="3">
         <v>-1.00288535955806</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="3">
         <v>-0.50769462311031799</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="3">
         <v>8.4069620611269796E-2</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="3">
         <v>-6.03904909844921</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="3">
         <v>1.93049590400193E-4</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="3">
         <v>-0.69787926099896702</v>
       </c>
-      <c r="G26" s="4">
+      <c r="G26" s="3">
         <v>-0.31752187211994398</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="3">
         <v>-0.96684277114304495</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="3">
         <v>0.14101799134637899</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="3">
         <v>-6.8562082423748096</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="3">
         <v>7.4215276548186701E-5</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="3">
         <v>-1.28585357379981</v>
       </c>
-      <c r="G27" s="4">
+      <c r="G27" s="3">
         <v>-0.64784385538455802</v>
       </c>
     </row>
@@ -1662,697 +1651,697 @@
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.44140625" customWidth="1"/>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="4" t="s">
+      <c r="A1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5">
-        <v>-0.52253281187205503</v>
-      </c>
-      <c r="C2" s="4">
-        <v>5.70285298883084E-2</v>
-      </c>
-      <c r="D2" s="4">
-        <v>-8.8175007335134907</v>
-      </c>
-      <c r="E2" s="4">
-        <v>2.15378843260811E-5</v>
-      </c>
-      <c r="F2" s="4">
-        <v>-0.63435712986840898</v>
-      </c>
-      <c r="G2" s="4">
-        <v>-0.37134107837430202</v>
+      <c r="B2" s="3">
+        <v>-0.503790953780059</v>
+      </c>
+      <c r="C2" s="3">
+        <v>5.8267877618851202E-2</v>
+      </c>
+      <c r="D2" s="3">
+        <v>-8.6664826028166306</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1.16158414861796E-5</v>
+      </c>
+      <c r="F2" s="3">
+        <v>-0.63678864440335603</v>
+      </c>
+      <c r="G2" s="3">
+        <v>-0.373166450970289</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5">
-        <v>-0.58881474953060198</v>
-      </c>
-      <c r="C3" s="4">
-        <v>6.8379728545350196E-2</v>
-      </c>
-      <c r="D3" s="4">
-        <v>-8.4136525507447697</v>
-      </c>
-      <c r="E3" s="4">
-        <v>3.0324397181909401E-5</v>
-      </c>
-      <c r="F3" s="4">
-        <v>-0.73300721428453597</v>
-      </c>
-      <c r="G3" s="4">
-        <v>-0.417639340705105</v>
+      <c r="B3" s="3">
+        <v>-0.57561060819490195</v>
+      </c>
+      <c r="C3" s="3">
+        <v>7.1291826947674705E-2</v>
+      </c>
+      <c r="D3" s="3">
+        <v>-8.0026681294975308</v>
+      </c>
+      <c r="E3" s="3">
+        <v>2.20759227868152E-5</v>
+      </c>
+      <c r="F3" s="3">
+        <v>-0.73179814838646295</v>
+      </c>
+      <c r="G3" s="3">
+        <v>-0.40925151442915703</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5">
-        <v>-1.7500224026120099</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0.107340283644699</v>
-      </c>
-      <c r="D4" s="4">
-        <v>-16.634814099870901</v>
-      </c>
-      <c r="E4" s="4">
-        <v>1.72387029925567E-7</v>
-      </c>
-      <c r="F4" s="4">
-        <v>-2.0331128018156299</v>
-      </c>
-      <c r="G4" s="4">
-        <v>-1.5380585258983099</v>
+      <c r="B4" s="3">
+        <v>-1.78417059468777</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.111926571039733</v>
+      </c>
+      <c r="D4" s="3">
+        <v>-15.638614446041901</v>
+      </c>
+      <c r="E4" s="3">
+        <v>7.8498900604743701E-8</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-2.0035719851428899</v>
+      </c>
+      <c r="G4" s="3">
+        <v>-1.4971809963729401</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5">
-        <v>-1.5039661484504001</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0.10288453039257101</v>
-      </c>
-      <c r="D5" s="4">
-        <v>-14.9149721933117</v>
-      </c>
-      <c r="E5" s="4">
-        <v>4.0270236635899102E-7</v>
-      </c>
-      <c r="F5" s="4">
-        <v>-1.7717720624609401</v>
-      </c>
-      <c r="G5" s="4">
-        <v>-1.29726775739333</v>
+      <c r="B5" s="3">
+        <v>-1.5329456248967499</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.102479283399924</v>
+      </c>
+      <c r="D5" s="3">
+        <v>-14.6339687692191</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1.3978191067917099E-7</v>
+      </c>
+      <c r="F5" s="3">
+        <v>-1.7315028777480099</v>
+      </c>
+      <c r="G5" s="3">
+        <v>-1.26785438778488</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="5">
-        <v>-0.91761150119939405</v>
-      </c>
-      <c r="C6" s="4">
-        <v>5.6050214164255603E-2</v>
-      </c>
-      <c r="D6" s="4">
-        <v>-16.888582727446298</v>
-      </c>
-      <c r="E6" s="4">
-        <v>1.5318420941736201E-7</v>
-      </c>
-      <c r="F6" s="4">
-        <v>-1.07586070444596</v>
-      </c>
-      <c r="G6" s="4">
-        <v>-0.81735665316225803</v>
+      <c r="B6" s="3">
+        <v>-0.94501847818830298</v>
+      </c>
+      <c r="C6" s="3">
+        <v>6.0450999707882098E-2</v>
+      </c>
+      <c r="D6" s="3">
+        <v>-15.3047143728744</v>
+      </c>
+      <c r="E6" s="3">
+        <v>9.4719661944392401E-8</v>
+      </c>
+      <c r="F6" s="3">
+        <v>-1.0619349460713501</v>
+      </c>
+      <c r="G6" s="3">
+        <v>-0.78843562209635198</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="5">
-        <v>-1.0850792485018901</v>
-      </c>
-      <c r="C7" s="4">
-        <v>7.2126381462809294E-2</v>
-      </c>
-      <c r="D7" s="4">
-        <v>-14.9053323515465</v>
-      </c>
-      <c r="E7" s="4">
-        <v>4.0472514593188999E-7</v>
-      </c>
-      <c r="F7" s="4">
-        <v>-1.24139142092815</v>
-      </c>
-      <c r="G7" s="4">
-        <v>-0.90874395310704503</v>
+      <c r="B7" s="3">
+        <v>-1.07565711034427</v>
+      </c>
+      <c r="C7" s="3">
+        <v>7.5829723693846995E-2</v>
+      </c>
+      <c r="D7" s="3">
+        <v>-14.118467677208001</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1.90677161477196E-7</v>
+      </c>
+      <c r="F7" s="3">
+        <v>-1.2421382555502301</v>
+      </c>
+      <c r="G7" s="3">
+        <v>-0.89906075033614397</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="5">
-        <v>-1.0320420194351301</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0.128084018748721</v>
-      </c>
-      <c r="D8" s="4">
-        <v>-8.0404863601943806</v>
-      </c>
-      <c r="E8" s="4">
-        <v>4.21091743195901E-5</v>
-      </c>
-      <c r="F8" s="4">
-        <v>-1.32522008259609</v>
-      </c>
-      <c r="G8" s="4">
-        <v>-0.73449552881985403</v>
+      <c r="B8" s="3">
+        <v>-1.0301060798322601</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.12981885847893401</v>
+      </c>
+      <c r="D8" s="3">
+        <v>-7.8940198356568496</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2.4619519607896501E-5</v>
+      </c>
+      <c r="F8" s="3">
+        <v>-1.31846330444944</v>
+      </c>
+      <c r="G8" s="3">
+        <v>-0.73112198330062905</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="5">
-        <v>-1.42585548921212</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0.132003031637277</v>
-      </c>
-      <c r="D9" s="4">
-        <v>-10.6619177235235</v>
-      </c>
-      <c r="E9" s="4">
-        <v>5.2498272942447801E-6</v>
-      </c>
-      <c r="F9" s="4">
-        <v>-1.7118049993873701</v>
-      </c>
-      <c r="G9" s="4">
-        <v>-1.10300592575727</v>
+      <c r="B9" s="3">
+        <v>-1.4075162526001099</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0.139477740347939</v>
+      </c>
+      <c r="D9" s="3">
+        <v>-10.0147241378621</v>
+      </c>
+      <c r="E9" s="3">
+        <v>3.5346780290981801E-6</v>
+      </c>
+      <c r="F9" s="3">
+        <v>-1.71235166233596</v>
+      </c>
+      <c r="G9" s="3">
+        <v>-1.0813105235779701</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="5">
-        <v>-1.7120798527741501</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0.20656738479155401</v>
-      </c>
-      <c r="D10" s="4">
-        <v>-7.8431005063475103</v>
-      </c>
-      <c r="E10" s="4">
-        <v>5.0346011219576899E-5</v>
-      </c>
-      <c r="F10" s="4">
-        <v>-2.0964740037811498</v>
-      </c>
-      <c r="G10" s="4">
-        <v>-1.1437835167258901</v>
+      <c r="B10" s="3">
+        <v>-1.6216422891201301</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0.205937922986557</v>
+      </c>
+      <c r="D10" s="3">
+        <v>-7.9162608149823104</v>
+      </c>
+      <c r="E10" s="3">
+        <v>2.40737430590429E-5</v>
+      </c>
+      <c r="F10" s="3">
+        <v>-2.09612225763316</v>
+      </c>
+      <c r="G10" s="3">
+        <v>-1.1643943624815001</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="5">
-        <v>-0.56116384477579395</v>
-      </c>
-      <c r="C11" s="4">
-        <v>5.6943689121905103E-2</v>
-      </c>
-      <c r="D11" s="4">
-        <v>-9.4039365196862903</v>
-      </c>
-      <c r="E11" s="4">
-        <v>1.3404252045642299E-5</v>
-      </c>
-      <c r="F11" s="4">
-        <v>-0.66680722028803996</v>
-      </c>
-      <c r="G11" s="4">
-        <v>-0.40418245511025302</v>
+      <c r="B11" s="3">
+        <v>-0.53652430994564804</v>
+      </c>
+      <c r="C11" s="3">
+        <v>5.7085737152173098E-2</v>
+      </c>
+      <c r="D11" s="3">
+        <v>-9.4808170056954992</v>
+      </c>
+      <c r="E11" s="3">
+        <v>5.5668012055584698E-6</v>
+      </c>
+      <c r="F11" s="3">
+        <v>-0.67035633676739004</v>
+      </c>
+      <c r="G11" s="3">
+        <v>-0.41208251838258197</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="5">
-        <v>-0.60269935069783398</v>
-      </c>
-      <c r="C12" s="4">
-        <v>5.7150491121600602E-2</v>
-      </c>
-      <c r="D12" s="4">
-        <v>-10.173934900967099</v>
-      </c>
-      <c r="E12" s="4">
-        <v>7.4617209663367804E-6</v>
-      </c>
-      <c r="F12" s="4">
-        <v>-0.71323464508482204</v>
-      </c>
-      <c r="G12" s="4">
-        <v>-0.449656107374102</v>
+      <c r="B12" s="3">
+        <v>-0.58277125268367203</v>
+      </c>
+      <c r="C12" s="3">
+        <v>5.9079767422258199E-2</v>
+      </c>
+      <c r="D12" s="3">
+        <v>-9.9098580777805605</v>
+      </c>
+      <c r="E12" s="3">
+        <v>3.8581583903254697E-6</v>
+      </c>
+      <c r="F12" s="3">
+        <v>-0.719119829473576</v>
+      </c>
+      <c r="G12" s="3">
+        <v>-0.45182439137214903</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="5">
-        <v>-0.74723026677037296</v>
-      </c>
-      <c r="C13" s="4">
-        <v>4.3108987775526901E-2</v>
-      </c>
-      <c r="D13" s="4">
-        <v>-16.676529781389402</v>
-      </c>
-      <c r="E13" s="4">
-        <v>1.6905279649423499E-7</v>
-      </c>
-      <c r="F13" s="4">
-        <v>-0.81831782255895502</v>
-      </c>
-      <c r="G13" s="4">
-        <v>-0.619498814409293</v>
+      <c r="B13" s="3">
+        <v>-0.71947138260508403</v>
+      </c>
+      <c r="C13" s="3">
+        <v>3.8715664837132499E-2</v>
+      </c>
+      <c r="D13" s="3">
+        <v>-18.524414727943199</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1.7830586432798201E-8</v>
+      </c>
+      <c r="F13" s="3">
+        <v>-0.80476595043490395</v>
+      </c>
+      <c r="G13" s="3">
+        <v>-0.62960411338727595</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="5">
-        <v>-1.00784479539697</v>
-      </c>
-      <c r="C14" s="4">
-        <v>7.7946855231644796E-2</v>
-      </c>
-      <c r="D14" s="4">
-        <v>-13.1321194548041</v>
-      </c>
-      <c r="E14" s="4">
-        <v>1.07551445355657E-6</v>
-      </c>
-      <c r="F14" s="4">
-        <v>-1.2033531845186101</v>
-      </c>
-      <c r="G14" s="4">
-        <v>-0.84386164353794602</v>
+      <c r="B14" s="3">
+        <v>-1.02268425869302</v>
+      </c>
+      <c r="C14" s="3">
+        <v>8.2361177296905397E-2</v>
+      </c>
+      <c r="D14" s="3">
+        <v>-12.0900501236602</v>
+      </c>
+      <c r="E14" s="3">
+        <v>7.2246305190009795E-7</v>
+      </c>
+      <c r="F14" s="3">
+        <v>-1.1820646889219399</v>
+      </c>
+      <c r="G14" s="3">
+        <v>-0.80943683460456295</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="5">
-        <v>-0.84259563933272497</v>
-      </c>
-      <c r="C15" s="4">
-        <v>8.3504804339612604E-2</v>
-      </c>
-      <c r="D15" s="4">
-        <v>-9.6812202073366809</v>
-      </c>
-      <c r="E15" s="4">
-        <v>1.08051365494253E-5</v>
-      </c>
-      <c r="F15" s="4">
-        <v>-1.00099082329891</v>
-      </c>
-      <c r="G15" s="4">
-        <v>-0.61586597506579199</v>
+      <c r="B15" s="3">
+        <v>-0.81079323871487197</v>
+      </c>
+      <c r="C15" s="3">
+        <v>8.5952485005854298E-2</v>
+      </c>
+      <c r="D15" s="3">
+        <v>-9.4742319200950593</v>
+      </c>
+      <c r="E15" s="3">
+        <v>5.5988177942765101E-6</v>
+      </c>
+      <c r="F15" s="3">
+        <v>-1.00877180667026</v>
+      </c>
+      <c r="G15" s="3">
+        <v>-0.61989574743765896</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="5">
-        <v>-1.3877153397395701</v>
-      </c>
-      <c r="C16" s="4">
-        <v>0.12987307504693699</v>
-      </c>
-      <c r="D16" s="4">
-        <v>-10.707099627479399</v>
-      </c>
-      <c r="E16" s="4">
-        <v>5.0853380246903997E-6</v>
-      </c>
-      <c r="F16" s="4">
-        <v>-1.69005180156459</v>
-      </c>
-      <c r="G16" s="4">
-        <v>-1.09107610534475</v>
+      <c r="B16" s="3">
+        <v>-1.3904913497439999</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.13551588823536001</v>
+      </c>
+      <c r="D16" s="3">
+        <v>-10.1379312336233</v>
+      </c>
+      <c r="E16" s="3">
+        <v>3.19226480057897E-6</v>
+      </c>
+      <c r="F16" s="3">
+        <v>-1.6804089932380399</v>
+      </c>
+      <c r="G16" s="3">
+        <v>-1.06729251874888</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="5">
-        <v>-2.1334699586950201</v>
-      </c>
-      <c r="C17" s="4">
-        <v>0.34335539430944501</v>
-      </c>
-      <c r="D17" s="4">
-        <v>-6.3117112886440596</v>
-      </c>
-      <c r="E17" s="4">
-        <v>2.2986983917904199E-4</v>
-      </c>
-      <c r="F17" s="4">
-        <v>-2.9589390774019901</v>
-      </c>
-      <c r="G17" s="4">
-        <v>-1.37538115915752</v>
+      <c r="B17" s="3">
+        <v>-2.1660399744893502</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.34588760330247598</v>
+      </c>
+      <c r="D17" s="3">
+        <v>-6.1965412522303298</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1.5952696889358001E-4</v>
+      </c>
+      <c r="F17" s="3">
+        <v>-2.9257589218326698</v>
+      </c>
+      <c r="G17" s="3">
+        <v>-1.3608546831650701</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="5">
-        <v>-0.58971650808602505</v>
-      </c>
-      <c r="C18" s="4">
-        <v>8.9622912863635606E-2</v>
-      </c>
-      <c r="D18" s="4">
-        <v>-6.4156706510232597</v>
-      </c>
-      <c r="E18" s="4">
-        <v>2.0567240241210001E-4</v>
-      </c>
-      <c r="F18" s="4">
-        <v>-0.78166189939102804</v>
-      </c>
-      <c r="G18" s="4">
-        <v>-0.36832028404585498</v>
+      <c r="B18" s="3">
+        <v>-0.57603562801806196</v>
+      </c>
+      <c r="C18" s="3">
+        <v>9.0309917867429701E-2</v>
+      </c>
+      <c r="D18" s="3">
+        <v>-6.5074619704546404</v>
+      </c>
+      <c r="E18" s="3">
+        <v>1.10488190214119E-4</v>
+      </c>
+      <c r="F18" s="3">
+        <v>-0.79198358365270405</v>
+      </c>
+      <c r="G18" s="3">
+        <v>-0.38339312850165702</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="5">
-        <v>-0.517079079002839</v>
-      </c>
-      <c r="C19" s="4">
-        <v>6.9036081095121604E-2</v>
-      </c>
-      <c r="D19" s="4">
-        <v>-7.6900781460435796</v>
-      </c>
-      <c r="E19" s="4">
-        <v>5.7968317044435401E-5</v>
-      </c>
-      <c r="F19" s="4">
-        <v>-0.690090347001727</v>
-      </c>
-      <c r="G19" s="4">
-        <v>-0.37169537003444703</v>
+      <c r="B19" s="3">
+        <v>-0.52892439215107301</v>
+      </c>
+      <c r="C19" s="3">
+        <v>6.5387942791659395E-2</v>
+      </c>
+      <c r="D19" s="3">
+        <v>-7.8229790465250604</v>
+      </c>
+      <c r="E19" s="3">
+        <v>2.6455747630807899E-5</v>
+      </c>
+      <c r="F19" s="3">
+        <v>-0.65944630950132199</v>
+      </c>
+      <c r="G19" s="3">
+        <v>-0.36361070320773903</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="5">
-        <v>-0.53118369958342704</v>
-      </c>
-      <c r="C20" s="4">
-        <v>2.75706877797844E-2</v>
-      </c>
-      <c r="D20" s="4">
-        <v>-19.108190426265001</v>
-      </c>
-      <c r="E20" s="4">
-        <v>5.82866654395885E-8</v>
-      </c>
-      <c r="F20" s="4">
-        <v>-0.59040407230982395</v>
-      </c>
-      <c r="G20" s="4">
-        <v>-0.46324783224861199</v>
+      <c r="B20" s="3">
+        <v>-0.52702850261561396</v>
+      </c>
+      <c r="C20" s="3">
+        <v>2.74459843717729E-2</v>
+      </c>
+      <c r="D20" s="3">
+        <v>-19.014130960875999</v>
+      </c>
+      <c r="E20" s="3">
+        <v>1.4173883629994099E-8</v>
+      </c>
+      <c r="F20" s="3">
+        <v>-0.58394867133169803</v>
+      </c>
+      <c r="G20" s="3">
+        <v>-0.45977441105839101</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="5">
-        <v>-1.5092784317056001</v>
-      </c>
-      <c r="C21" s="4">
-        <v>0.13681607218786401</v>
-      </c>
-      <c r="D21" s="4">
-        <v>-11.176907570944101</v>
-      </c>
-      <c r="E21" s="4">
-        <v>3.6774482094718198E-6</v>
-      </c>
-      <c r="F21" s="4">
-        <v>-1.84467902129098</v>
-      </c>
-      <c r="G21" s="4">
-        <v>-1.2136821648357601</v>
+      <c r="B21" s="3">
+        <v>-1.52760392501248</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0.13897105360451101</v>
+      </c>
+      <c r="D21" s="3">
+        <v>-10.732588382588199</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1.98061603297255E-6</v>
+      </c>
+      <c r="F21" s="3">
+        <v>-1.80589347976488</v>
+      </c>
+      <c r="G21" s="3">
+        <v>-1.17714475109876</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="5">
-        <v>-0.90214523845726202</v>
-      </c>
-      <c r="C22" s="4">
-        <v>0.42546109079813399</v>
-      </c>
-      <c r="D22" s="4">
-        <v>-1.9644869382812999</v>
-      </c>
-      <c r="E22" s="4">
-        <v>8.5065864415276596E-2</v>
-      </c>
-      <c r="F22" s="4">
-        <v>-1.8169277903688199</v>
-      </c>
-      <c r="G22" s="4">
-        <v>0.14530227912912499</v>
+      <c r="B22" s="3">
+        <v>-0.83612033855998502</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0.42249776065635303</v>
+      </c>
+      <c r="D22" s="3">
+        <v>-1.96550590058053</v>
+      </c>
+      <c r="E22" s="3">
+        <v>8.0924920381673704E-2</v>
+      </c>
+      <c r="F22" s="3">
+        <v>-1.7861781770870899</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0.12533449398284799</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="5">
-        <v>-1.5947580894711899</v>
-      </c>
-      <c r="C23" s="4">
-        <v>0.13737563665732999</v>
-      </c>
-      <c r="D23" s="4">
-        <v>-11.6581257552461</v>
-      </c>
-      <c r="E23" s="4">
-        <v>2.67130842449341E-6</v>
-      </c>
-      <c r="F23" s="4">
-        <v>-1.9183312340662499</v>
-      </c>
-      <c r="G23" s="4">
-        <v>-1.2847536616500299</v>
+      <c r="B23" s="3">
+        <v>-1.6001173391912</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0.14310951294836</v>
+      </c>
+      <c r="D23" s="3">
+        <v>-10.9301843414296</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1.6987020831407701E-6</v>
+      </c>
+      <c r="F23" s="3">
+        <v>-1.8879495673184801</v>
+      </c>
+      <c r="G23" s="3">
+        <v>-1.2404771477570899</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="5">
-        <v>-1.40384996280401</v>
-      </c>
-      <c r="C24" s="4">
-        <v>0.110857787415499</v>
-      </c>
-      <c r="D24" s="4">
-        <v>-12.607425229393</v>
-      </c>
-      <c r="E24" s="4">
-        <v>1.4702821305984501E-6</v>
-      </c>
-      <c r="F24" s="4">
-        <v>-1.6532697821365701</v>
-      </c>
-      <c r="G24" s="4">
-        <v>-1.1419927497371201</v>
+      <c r="B24" s="3">
+        <v>-1.39755782045907</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0.111396366432383</v>
+      </c>
+      <c r="D24" s="3">
+        <v>-12.386854964553001</v>
+      </c>
+      <c r="E24" s="3">
+        <v>5.8736626440664802E-7</v>
+      </c>
+      <c r="F24" s="3">
+        <v>-1.63184672281084</v>
+      </c>
+      <c r="G24" s="3">
+        <v>-1.12785454634142</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="5">
-        <v>-1.2207771640338001</v>
-      </c>
-      <c r="C25" s="4">
-        <v>0.108139762607186</v>
-      </c>
-      <c r="D25" s="4">
-        <v>-10.9064725208976</v>
-      </c>
-      <c r="E25" s="4">
-        <v>4.4251006649485804E-6</v>
-      </c>
-      <c r="F25" s="4">
-        <v>-1.42879408904384</v>
-      </c>
-      <c r="G25" s="4">
-        <v>-0.93005260953950097</v>
+      <c r="B25" s="3">
+        <v>-1.1788745227473101</v>
+      </c>
+      <c r="C25" s="3">
+        <v>0.111938806837402</v>
+      </c>
+      <c r="D25" s="3">
+        <v>-10.375204811876801</v>
+      </c>
+      <c r="E25" s="3">
+        <v>2.6312394799106901E-6</v>
+      </c>
+      <c r="F25" s="3">
+        <v>-1.4146112210174699</v>
+      </c>
+      <c r="G25" s="3">
+        <v>-0.90816487365284204</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="5">
-        <v>-0.50905610951238001</v>
-      </c>
-      <c r="C26" s="4">
-        <v>0.10374089843296699</v>
-      </c>
-      <c r="D26" s="4">
-        <v>-4.5663668409758804</v>
-      </c>
-      <c r="E26" s="4">
-        <v>1.8345121808805199E-3</v>
-      </c>
-      <c r="F26" s="4">
-        <v>-0.71294593943356699</v>
-      </c>
-      <c r="G26" s="4">
-        <v>-0.23449205788113101</v>
+      <c r="B26" s="3">
+        <v>-0.47498173216436002</v>
+      </c>
+      <c r="C26" s="3">
+        <v>0.10134110985362201</v>
+      </c>
+      <c r="D26" s="3">
+        <v>-4.8171967870930503</v>
+      </c>
+      <c r="E26" s="3">
+        <v>9.5067805668044804E-4</v>
+      </c>
+      <c r="F26" s="3">
+        <v>-0.71742958632860498</v>
+      </c>
+      <c r="G26" s="3">
+        <v>-0.25893055124602199</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="5">
-        <v>-0.978668873912933</v>
-      </c>
-      <c r="C27" s="4">
-        <v>0.152230107215587</v>
-      </c>
-      <c r="D27" s="4">
-        <v>-6.0911635101449502</v>
-      </c>
-      <c r="E27" s="4">
-        <v>2.92304745044514E-4</v>
-      </c>
-      <c r="F27" s="4">
-        <v>-1.2783017309587501</v>
-      </c>
-      <c r="G27" s="4">
-        <v>-0.57621521747531901</v>
+      <c r="B27" s="3">
+        <v>-0.92763206000377596</v>
+      </c>
+      <c r="C27" s="3">
+        <v>0.154677380630416</v>
+      </c>
+      <c r="D27" s="3">
+        <v>-5.9679244064544301</v>
+      </c>
+      <c r="E27" s="3">
+        <v>2.1063802973090101E-4</v>
+      </c>
+      <c r="F27" s="3">
+        <v>-1.2730074595066601</v>
+      </c>
+      <c r="G27" s="3">
+        <v>-0.57319837047474098</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B28" s="5">
-        <v>-1.7864189127020098E-2</v>
-      </c>
-      <c r="C28" s="4">
-        <v>0.23364274468131699</v>
-      </c>
-      <c r="D28" s="4">
-        <v>1.8145425964308699</v>
-      </c>
-      <c r="E28" s="4">
-        <v>0.107143364149034</v>
-      </c>
-      <c r="F28" s="4">
-        <v>-0.114826422824296</v>
-      </c>
-      <c r="G28" s="4">
-        <v>0.96273584796684097</v>
+      <c r="A28" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="3">
+        <v>0.40393846470533601</v>
+      </c>
+      <c r="C28" s="3">
+        <v>0.18047316860680301</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0.95019247439174304</v>
+      </c>
+      <c r="E28" s="3">
+        <v>0.36683134844460902</v>
+      </c>
+      <c r="F28" s="3">
+        <v>-0.23677442441695101</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0.57974291769658504</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" s="5">
-        <v>1.6770402815752601</v>
-      </c>
-      <c r="C29" s="4">
-        <v>0.34423056842465599</v>
-      </c>
-      <c r="D29" s="4">
-        <v>4.7189812041628496</v>
-      </c>
-      <c r="E29" s="4">
-        <v>1.50414008319298E-3</v>
-      </c>
-      <c r="F29" s="4">
-        <v>0.83062046804330703</v>
-      </c>
-      <c r="G29" s="4">
-        <v>2.4182146965451801</v>
+      <c r="A29" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="3">
+        <v>1.61755060940589</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0.348286529548122</v>
+      </c>
+      <c r="D29" s="3">
+        <v>4.81318942155045</v>
+      </c>
+      <c r="E29" s="3">
+        <v>9.5599463536777895E-4</v>
+      </c>
+      <c r="F29" s="3">
+        <v>0.88849017216612503</v>
+      </c>
+      <c r="G29" s="3">
+        <v>2.46424790721295</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="5">
-        <v>3.76457388476008E-4</v>
-      </c>
-      <c r="C30" s="4">
-        <v>2.8837126913632701E-3</v>
-      </c>
-      <c r="D30" s="4">
-        <v>0.86046771219048501</v>
-      </c>
-      <c r="E30" s="4">
-        <v>0.41457341921011898</v>
-      </c>
-      <c r="F30" s="4">
-        <v>-4.1685117288724101E-3</v>
-      </c>
-      <c r="G30" s="4">
-        <v>9.1311950531764493E-3</v>
+      <c r="A30" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="3">
+        <v>2.4024105994670799E-3</v>
+      </c>
+      <c r="C30" s="3">
+        <v>3.47529214796145E-3</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.218050070226777</v>
+      </c>
+      <c r="E30" s="3">
+        <v>0.83225384098979005</v>
+      </c>
+      <c r="F30" s="3">
+        <v>-7.10386932840579E-3</v>
+      </c>
+      <c r="G30" s="3">
+        <v>8.6194447222489208E-3</v>
       </c>
     </row>
   </sheetData>
@@ -2365,627 +2354,627 @@
   <dimension ref="A1:G27"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.5546875" customWidth="1"/>
+    <col min="1" max="1" width="17.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3">
         <v>-0.68602943416995599</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>8.0635037186269298E-2</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>-8.5078330476267805</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>1.34931131924825E-5</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <v>-0.86843856111337503</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="3">
         <v>-0.50362030722653806</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>-0.74015230759494599</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>9.4411981683629007E-2</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>-7.8396014403676801</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>2.60130184722503E-5</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>-0.95372704821454002</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>-0.52657756697535096</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>-2.02464139941014</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>0.159778821269735</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>-12.6715254457422</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>4.83593539550033E-7</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>-2.3860862044089202</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>-1.66319659441135</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>-1.7922398739029</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>0.13122033924717999</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>-13.6582475261465</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>2.5384976997878799E-7</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>-2.0890809042357201</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="3">
         <v>-1.49539884357009</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>-1.039658019165</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>9.7164807092031E-2</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>-10.699944252246301</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>2.0319799562029202E-6</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>-1.2594600835001499</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>-0.81985595482985796</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>-1.2746966554175501</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>6.5361764126705593E-2</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>-19.502176424530401</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>1.1338726488980001E-8</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <v>-1.42255523830991</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="3">
         <v>-1.1268380725252001</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>-1.18399855662465</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>0.133662157307294</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>-8.8581434003238098</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>9.7212371972748092E-6</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <v>-1.4863633631724</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="3">
         <v>-0.88163375007689104</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>-1.5849396832668901</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>0.14513723885008201</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>-10.9202827325662</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>1.71172354240193E-6</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>-1.9132629277203601</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <v>-1.25661643881342</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="3">
         <v>-1.8938419230832499</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>0.234770840910489</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>-8.0667680694014194</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>2.0711477039501199E-5</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>-2.42493046246507</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>-1.3627533837014301</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="3">
         <v>-0.734600687282701</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>8.6036301774082294E-2</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>-8.5382643388327608</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>1.3108631328789799E-5</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>-0.92922832360160901</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <v>-0.539973050963793</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="3">
         <v>-0.818995523351293</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>0.101102927879743</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>-8.1006113326950508</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>2.0028630664924599E-5</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>-1.0477062358343201</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>-0.59028481086826301</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="3">
         <v>-1.0032447513567</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>0.104029127924561</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>-9.6438831255437201</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>4.8349031945516696E-6</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>-1.2385749882309001</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="3">
         <v>-0.76791451448250603</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="3">
         <v>-1.2519628396962299</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>9.0236449728195098E-2</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>-13.8742475293223</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <v>2.2170543078441599E-7</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="3">
         <v>-1.45609187079434</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="3">
         <v>-1.04783380859811</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="3">
         <v>-1.06253183574225</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>0.14005283438664401</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="3">
         <v>-7.5866499981636997</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>3.3731535437046798E-5</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="3">
         <v>-1.37935335822019</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <v>-0.74571031326431603</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="3">
         <v>-1.6490114367041</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <v>0.1469610057312</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>-11.2207413694503</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <v>1.3612909603377701E-6</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="3">
         <v>-1.98146032847097</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="3">
         <v>-1.31656254493724</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="3">
         <v>-2.31060822109347</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>0.30037997702170399</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>-7.6922844325489796</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <v>3.0238981895011602E-5</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="3">
         <v>-2.9901149376742802</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="3">
         <v>-1.63110150451267</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="3">
         <v>-0.63039029732847296</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="3">
         <v>6.8422949172690206E-2</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>-9.2131412771678995</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <v>7.0473801833391201E-6</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="3">
         <v>-0.78517376189925203</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="3">
         <v>-0.475606832757695</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="3">
         <v>-0.49917409175785799</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="3">
         <v>4.9198451950983303E-2</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>-10.1461341152601</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <v>3.1708017843739501E-6</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="3">
         <v>-0.61046872223735904</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="3">
         <v>-0.38787946127835798</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="3">
         <v>-0.67246760926448101</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="3">
         <v>4.7410174176853302E-2</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>-14.1840358307056</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <v>1.8318795705836699E-7</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="3">
         <v>-0.77971687436815995</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="3">
         <v>-0.56521834416080197</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="3">
         <v>-1.80577643018178</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="3">
         <v>0.16577580674752199</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <v>-10.892882777111099</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <v>1.7483346043758201E-6</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="3">
         <v>-2.1807873588343401</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="3">
         <v>-1.43076550152922</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="3">
         <v>-1.0766642130533199</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="3">
         <v>0.36592888257106798</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="3">
         <v>-2.94227721378134</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="3">
         <v>1.6425816136227601E-2</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="3">
         <v>-1.9044528558362099</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="3">
         <v>-0.248875570270436</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="3">
         <v>-1.8489277231371299</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="3">
         <v>0.158605950994889</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <v>-11.6573666469597</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="3">
         <v>9.8510624271209307E-7</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="3">
         <v>-2.2077193112426401</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="3">
         <v>-1.49013613503163</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="3">
         <v>-1.65382092616869</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="3">
         <v>0.12621505333222399</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="3">
         <v>-13.103198727139899</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <v>3.6280273001230098E-7</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="3">
         <v>-1.9393392131171401</v>
       </c>
-      <c r="G24" s="4">
+      <c r="G24" s="3">
         <v>-1.36830263922024</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="3">
         <v>-1.4170496102576999</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <v>0.148965986928393</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <v>-9.5125715572835201</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="3">
         <v>5.4152151140347104E-6</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="3">
         <v>-1.75403408460107</v>
       </c>
-      <c r="G25" s="4">
+      <c r="G25" s="3">
         <v>-1.0800651359143301</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="3">
         <v>-0.645195741987445</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="3">
         <v>8.6633788024013905E-2</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="3">
         <v>-7.4473915628461702</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="3">
         <v>3.9028701276067903E-5</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="3">
         <v>-0.84117498610630903</v>
       </c>
-      <c r="G26" s="4">
+      <c r="G26" s="3">
         <v>-0.44921649786857998</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="3">
         <v>-1.1043438900201801</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="3">
         <v>0.16743213102649801</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="3">
         <v>-6.5957703772247296</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="3">
         <v>9.9759895200627593E-5</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="3">
         <v>-1.4831016845043401</v>
       </c>
-      <c r="G27" s="4">
+      <c r="G27" s="3">
         <v>-0.72558609553602404</v>
       </c>
     </row>
@@ -2999,650 +2988,650 @@
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.77734375" customWidth="1"/>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2">
+      <c r="A2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="3">
         <v>6.8442564552467502</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>3.1906124345812303E-2</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>214.50571088146901</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>5.2914369015886698E-18</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <v>6.7718692165450198</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="3">
         <v>6.9162225519970404</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>-0.96096594040446104</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>4.6134177590189597E-2</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>-20.8252410601775</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>6.3542331518881399E-9</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>-1.0651181297141901</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>-0.85639260914328297</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>-0.43402255419591801</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>5.9074291114912997E-2</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>-7.34349875441296</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>4.3573754109954601E-5</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>-0.56744731400301895</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>-0.30017665243736602</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>-1.0065367748427301</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>0.100975974087057</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>-9.9659964953583504</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>3.68111074075098E-6</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>-1.2347497269185601</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="3">
         <v>-0.77790268081544101</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>-2.5722879220431598</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>9.7999408696419599E-2</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>-26.245845615611401</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>8.1707372801826305E-10</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>-2.7937674154000298</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>-2.3503872867348399</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>0.25487109150482601</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>4.1971261474621997E-2</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>6.0775314707847796</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>1.8420438500469299E-4</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <v>0.16013607270406</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="3">
         <v>0.35002725225704501</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>-0.90108037982635403</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>5.2004302980971799E-2</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>-17.3229859302268</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>3.2118410987055701E-8</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <v>-1.01851171533536</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="3">
         <v>-0.78322790236589501</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>-1.6094098412137801</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>9.3211767983874094E-2</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>-17.2639067474447</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>3.3094231478898303E-8</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>-1.82005893883986</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <v>-1.3983396016362499</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="3">
         <v>-2.23730001977715</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>0.10404638155745</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>-21.500886578801399</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>4.7918432031348297E-9</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>-2.4724587161048501</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>-2.0017201814980101</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="3">
         <v>-1.8172437292560599</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>0.17431001310771399</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>-10.424146759472199</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>2.5296005577981402E-6</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>-2.2113498029794001</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <v>-1.42271651358127</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="3">
         <v>1.17878238242509</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>6.0309902699858198E-2</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>19.548911548875601</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>1.11020961245208E-8</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>1.0425624750206699</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>1.3154234317809701</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="3">
         <v>0.65201605281182295</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>6.3181445056535904E-2</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>10.323072275474599</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>2.7444838013685599E-6</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>0.50930026529696604</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="3">
         <v>0.79515298227813402</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="3">
         <v>0.10514820412341599</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>7.6930380321318895E-2</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>1.3695340470057</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <v>0.20403007136257101</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="3">
         <v>-6.8669835781517696E-2</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="3">
         <v>0.279387385979806</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="3">
         <v>-1.0319333400577499</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>7.3393193819919794E-2</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="3">
         <v>-14.0574720268135</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>1.97949269397177E-7</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="3">
         <v>-1.19774970818239</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <v>-0.86569582998165395</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="3">
         <v>0.67648421428665895</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <v>9.7537942937916997E-2</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>6.9377594490905699</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <v>6.7760693676759698E-5</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="3">
         <v>0.45604862900077903</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="3">
         <v>0.89734094152400201</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="3">
         <v>-1.9283884570794001</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>0.121959437998914</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>-15.8099932054529</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <v>7.1387768534666595E-8</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="3">
         <v>-2.2040693023437599</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="3">
         <v>-1.65228646986359</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="3">
         <v>-1.41154374670083</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="3">
         <v>0.243764727014083</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>-5.78973501627069</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <v>2.6283526733988E-4</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="3">
         <v>-1.96276729897756</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="3">
         <v>-0.85989905247264697</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="3">
         <v>-1.2368272006821099</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="3">
         <v>4.0300286692318603E-2</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>-30.6850578793049</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <v>2.0306060665379301E-10</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="3">
         <v>-1.32778221191023</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="3">
         <v>-1.1454510475025299</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="3">
         <v>-2.33542460306685</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="3">
         <v>4.13225355600167E-2</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>-56.511876641729003</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <v>8.5627512656923501E-13</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="3">
         <v>-2.4286921018932</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="3">
         <v>-2.24173596228905</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="3">
         <v>-0.49149114095396601</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="3">
         <v>3.6599199425131297E-2</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <v>-13.4232600082748</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <v>2.94796258409801E-7</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="3">
         <v>-0.574073711110478</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="3">
         <v>-0.40848742884599698</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="3">
         <v>-0.135467924196604</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="3">
         <v>0.141081459277244</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="3">
         <v>-0.95871813287014795</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="3">
         <v>0.36274573446429198</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="3">
         <v>-0.45440578686291699</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="3">
         <v>0.183891080421166</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="3">
         <v>-8.7101233428981503E-2</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="3">
         <v>0.32061987206286302</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <v>-0.27100834983870298</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="3">
         <v>0.79249773048580296</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="3">
         <v>-0.81218320257570298</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="3">
         <v>0.63840187766919798</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="3">
         <v>-0.36322908828285499</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="3">
         <v>0.12951727648662401</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="3">
         <v>-2.8028578669550401</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <v>2.0616160249642398E-2</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="3">
         <v>-0.65600695201745796</v>
       </c>
-      <c r="G24" s="4">
+      <c r="G24" s="3">
         <v>-7.0030082596793303E-2</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="3">
         <v>-1.5701494349789999</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <v>9.4144161766335305E-2</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <v>-16.6759025153343</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="3">
         <v>4.4819282563029401E-8</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="3">
         <v>-1.78290775387862</v>
       </c>
-      <c r="G25" s="4">
+      <c r="G25" s="3">
         <v>-1.35696997412793</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="3">
         <v>-3.1077436305302499</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="3">
         <v>9.3817726637638599E-2</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="3">
         <v>-33.123090602664597</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="3">
         <v>1.02607137811405E-10</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="3">
         <v>-3.3197635018653</v>
       </c>
-      <c r="G26" s="4">
+      <c r="G26" s="3">
         <v>-2.8953026172437499</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="3">
         <v>0.96433365522347902</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="3">
         <v>6.4780604389535507E-2</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="3">
         <v>14.889398382257401</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="3">
         <v>1.2029738881734401E-7</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="3">
         <v>0.81800031796902395</v>
       </c>
-      <c r="G27" s="4">
+      <c r="G27" s="3">
         <v>1.1110881344293899</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="3">
         <v>-0.62964370839858697</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="3">
         <v>0.123753069182045</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D28" s="3">
         <v>-5.0862022379173002</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E28" s="3">
         <v>6.5729596687736898E-4</v>
       </c>
-      <c r="F28" s="4">
+      <c r="F28" s="3">
         <v>-0.90938202929127898</v>
       </c>
-      <c r="G28" s="4">
+      <c r="G28" s="3">
         <v>-0.34948424555442797</v>
       </c>
     </row>

</xml_diff>